<commit_message>
Further added rock type mapping for Xianshuihe, Australia, Thailand and USGS Database. Missing Argonne due to not being able to finde rock type data
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Southern_Thailand_Parsed.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Southern_Thailand_Parsed.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a36cc37384f3e2/SPEICHER/Hochschule/7. Semester/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55588F82-2EC9-43C8-A740-3941A23563AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{55588F82-2EC9-43C8-A740-3941A23563AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2971EC4-E18D-4CEB-A767-9E1FD75B0C39}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4260" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="61">
   <si>
-    <t>Surface temperature (°C)</t>
-  </si>
-  <si>
     <t>East (m)</t>
   </si>
   <si>
@@ -203,6 +200,9 @@
   </si>
   <si>
     <t>HCO3_mg-L</t>
+  </si>
+  <si>
+    <t>Surface_temperature</t>
   </si>
 </sst>
 </file>
@@ -574,77 +574,78 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="3" max="3" width="25.140625" customWidth="1"/>
     <col min="9" max="9" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="T1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>50</v>
@@ -703,10 +704,10 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>65</v>
@@ -765,10 +766,10 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4">
         <v>40</v>
@@ -827,10 +828,10 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5">
         <v>45</v>
@@ -889,10 +890,10 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>50</v>
@@ -951,10 +952,10 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7">
         <v>46</v>
@@ -1013,10 +1014,10 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8">
         <v>75</v>
@@ -1075,10 +1076,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9">
         <v>45</v>
@@ -1137,10 +1138,10 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C10">
         <v>40</v>
@@ -1199,10 +1200,10 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C11">
         <v>60</v>
@@ -1261,10 +1262,10 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12">
         <v>41</v>
@@ -1323,10 +1324,10 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13">
         <v>42</v>
@@ -1385,10 +1386,10 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14">
         <v>53</v>
@@ -1447,10 +1448,10 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15">
         <v>70</v>
@@ -1509,10 +1510,10 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16">
         <v>56</v>
@@ -1571,10 +1572,10 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C17">
         <v>62</v>
@@ -1633,10 +1634,10 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C18">
         <v>78</v>
@@ -1695,10 +1696,10 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C19">
         <v>55</v>
@@ -1757,10 +1758,10 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C20">
         <v>45</v>
@@ -1819,10 +1820,10 @@
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C21">
         <v>45</v>
@@ -1881,10 +1882,10 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C22">
         <v>47</v>
@@ -1943,10 +1944,10 @@
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23">
         <v>45</v>
@@ -2005,10 +2006,10 @@
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C24">
         <v>47</v>
@@ -2067,10 +2068,10 @@
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25">
         <v>47</v>
@@ -2129,10 +2130,10 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C26">
         <v>52</v>
@@ -2168,7 +2169,7 @@
         <v>29.2</v>
       </c>
       <c r="N26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O26">
         <v>0.02</v>
@@ -2191,10 +2192,10 @@
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C27">
         <v>50</v>
@@ -2253,10 +2254,10 @@
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C28">
         <v>57</v>
@@ -2315,10 +2316,10 @@
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C29">
         <v>46</v>
@@ -2377,10 +2378,10 @@
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C30">
         <v>50</v>
@@ -2439,10 +2440,10 @@
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C31">
         <v>41</v>
@@ -2501,10 +2502,10 @@
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C32">
         <v>80</v>

</xml_diff>

<commit_message>
Extracting Ion-charges for better comprehension. Will try another Approach - only with main Ions
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Southern_Thailand_Parsed.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Southern_Thailand_Parsed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a36cc37384f3e2/SPEICHER/Hochschule/7. Semester/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{55588F82-2EC9-43C8-A740-3941A23563AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2971EC4-E18D-4CEB-A767-9E1FD75B0C39}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{55588F82-2EC9-43C8-A740-3941A23563AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A86C1B2-8583-4FEF-A8DC-ABE5D07FE1F7}"/>
   <bookViews>
-    <workbookView xWindow="4260" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -175,9 +175,6 @@
     <t>Hot_spring</t>
   </si>
   <si>
-    <t>Na_mg-L)</t>
-  </si>
-  <si>
     <t>K_mg-L</t>
   </si>
   <si>
@@ -203,6 +200,9 @@
   </si>
   <si>
     <t>Surface_temperature</t>
+  </si>
+  <si>
+    <t>Na_mg-L</t>
   </si>
 </sst>
 </file>
@@ -586,7 +586,7 @@
         <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -607,34 +607,34 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="Q1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="T1" t="s">
         <v>48</v>

</xml_diff>